<commit_message>
Update rental rates and long-term Avito prices for 2026-10-02
</commit_message>
<xml_diff>
--- a/stroyrent39-avito-19-2026-09-30.xlsx
+++ b/stroyrent39-avito-19-2026-09-30.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" r:id="Rd790d10789e141e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объявления" sheetId="2" r:id="Rbe4d2994ea114423"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Справочники" sheetId="3" r:id="Rcf435e8f50ce40ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" r:id="Rc94d02b866344408"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объявления" sheetId="2" r:id="Rbc3b52e0403640de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Справочники" sheetId="3" r:id="Rab715bfd40364489"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="Instructions" localSheetId="0">Инструкция!$1:$50</x:definedName>
@@ -752,15 +752,6 @@
   <x:si>
     <x:r>
       <x:rPr>
-        <x:color rgb="FFF28D00"/>
-        <x:family val="2"/>
-      </x:rPr>
-      <x:t xml:space="preserve">Обязательный</x:t>
-    </x:r>
-  </x:si>
-  <x:si>
-    <x:r>
-      <x:rPr>
         <x:sz val="1100"/>
         <x:color rgb="FF000000"/>
       </x:rPr>
@@ -783,11 +774,6 @@
         <x:color rgb="FF000000"/>
       </x:rPr>
       <x:t xml:space="preserve">Текст</x:t>
-    </x:r>
-  </x:si>
-  <x:si>
-    <x:r>
-      <x:t xml:space="preserve">Одно значение из выпадающего списка в ячейке</x:t>
     </x:r>
   </x:si>
   <x:si>
@@ -1317,13 +1303,13 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="R486f9d04a0fd4060"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="R352e647d5f5e48ca"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="Rd40c747511844253"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="Rfc53c3b08e544884"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="Rc568381b9f88411e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="R5e14228fa72a4d4d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="R6b4f1691aff044cc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="Rdf2c534d021a4a85"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="Re48645af10114a50"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="Rb97e80e103514a53"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="R514e0e2dd4f64d51"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="R47afc86d016e4553"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="R675692cdb59d41a2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="Rd44b8462277e4be5"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1410,13 +1396,13 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="H3" s="6" t="s">
-        <x:v>49</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="I3" s="6" t="s">
-        <x:v>49</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="J3" s="6" t="s">
-        <x:v>49</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="K3" t="str">
         <x:v>Необязательный</x:v>
@@ -1424,37 +1410,37 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B4" s="5" t="s">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="B4" s="5" t="s">
+      <x:c r="C4" s="5" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D4" s="5" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="E4" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="C4" s="5" t="s">
+      <x:c r="F4" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="D4" s="5" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E4" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="F4" t="s">
-        <x:v>52</x:v>
-      </x:c>
       <x:c r="G4" s="5" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="H4" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="I4" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="J4" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="K4" t="str">
-        <x:v>Целое число, ₽ за первые сутки</x:v>
+        <x:v>Целое число, ₽/сутки по минимальному тарифу; срок указан в описании</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="285" customHeight="1">
@@ -1478,8 +1464,10 @@
 1–3 суток — 2 100 ₽/сутки
 4–7 суток — 1 650 ₽/сутки
 от 8 суток — 1 600 ₽/сутки
+Цена в объявлении — 1 600 ₽/сутки при аренде от 8 суток.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Топливо в стоимость аренды не входит.
+Расходные материалы оплачиваются отдельно.
 Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
       </x:c>
       <x:c r="G5" s="8" t="str">
@@ -1495,7 +1483,7 @@
         <x:v>Строительное оборудование</x:v>
       </x:c>
       <x:c r="K5" s="10" t="n">
-        <x:v>2100</x:v>
+        <x:v>1600</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="285" customHeight="1">
@@ -1519,8 +1507,10 @@
 1–2 суток — 1 800 ₽/сутки
 3–7 суток — 1 300 ₽/сутки
 от 8 суток — 1 250 ₽/сутки
+Цена в объявлении — 1 250 ₽/сутки при аренде от 8 суток.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Топливо в стоимость аренды не входит.
+Расходные материалы оплачиваются отдельно.
 Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
       </x:c>
       <x:c r="G6" s="8" t="str">
@@ -1536,7 +1526,7 @@
         <x:v>Строительное оборудование</x:v>
       </x:c>
       <x:c r="K6" s="10" t="n">
-        <x:v>1800</x:v>
+        <x:v>1250</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="285" customHeight="1">
@@ -1560,8 +1550,10 @@
 1–3 суток — 1 300 ₽/сутки
 4–7 суток — 1 050 ₽/сутки
 от 8 суток — 950 ₽/сутки
+Цена в объявлении — 950 ₽/сутки при аренде от 8 суток.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Топливо в стоимость аренды не входит.
+Расходные материалы оплачиваются отдельно.
 Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
       </x:c>
       <x:c r="G7" s="8" t="str">
@@ -1577,7 +1569,7 @@
         <x:v>Строительное оборудование</x:v>
       </x:c>
       <x:c r="K7" s="10" t="n">
-        <x:v>1300</x:v>
+        <x:v>950</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="285" customHeight="1">
@@ -1598,11 +1590,13 @@
         <x:v>Прокат виброплиты CHAMPION PC1151FT в Калининграде и области. Бензиновая виброплита для уплотнения песка, гравия и брусчатки. Коврик для работы по плитке — бесплатно в комплекте с арендой.
 Характеристики: центробежная сила — 25 кН; размер плиты — 500 × 580 мм; глубина уплотнения — 350 мм; вес — 103,4 кг.
 Стоимость аренды за сутки:
-1–2 суток — 1 700 ₽/сутки
-3–7 суток — 1 550 ₽/сутки
-от 8 суток — 1 450 ₽/сутки
+1–2 суток — 2 200 ₽/сутки
+3–7 суток — 2 000 ₽/сутки
+от 8 суток — 1 900 ₽/сутки
+Цена в объявлении — 1 900 ₽/сутки при аренде от 8 суток.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Топливо в стоимость аренды не входит.
+Расходные материалы оплачиваются отдельно.
 Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
       </x:c>
       <x:c r="G8" s="8" t="str">
@@ -1618,7 +1612,7 @@
         <x:v>Строительное оборудование</x:v>
       </x:c>
       <x:c r="K8" s="10" t="n">
-        <x:v>1700</x:v>
+        <x:v>1900</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="285" customHeight="1">
@@ -1639,11 +1633,13 @@
         <x:v>Прокат реверсивной виброплиты CHAMPION PC1645RH в Калининграде и области. Реверсивная бензиновая виброплита для уплотнения песка, гравия и брусчатки. Обратный ход упрощает маневрирование. Коврик для работы по плитке — бесплатно в комплекте с арендой.
 Характеристики: центробежная сила — 30,5 кН; размер плиты — 730 × 450 мм; глубина уплотнения — 500 мм; вес — 152 кг.
 Стоимость аренды за сутки:
-1 сутки — 1 950 ₽/сутки
-2–7 суток — 1 700 ₽/сутки
-от 8 суток — 1 650 ₽/сутки
+1 сутки — 2 500 ₽/сутки
+2–7 суток — 2 200 ₽/сутки
+от 8 суток — 2 150 ₽/сутки
+Цена в объявлении — 2 150 ₽/сутки при аренде от 8 суток.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Топливо в стоимость аренды не входит.
+Расходные материалы оплачиваются отдельно.
 Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
       </x:c>
       <x:c r="G9" s="8" t="str">
@@ -1659,7 +1655,7 @@
         <x:v>Строительное оборудование</x:v>
       </x:c>
       <x:c r="K9" s="10" t="n">
-        <x:v>1950</x:v>
+        <x:v>2150</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="285" customHeight="1">
@@ -1683,7 +1679,9 @@
 1–2 суток — 1 200 ₽/сутки
 3–7 суток — 1 000 ₽/сутки
 от 8 суток — 900 ₽/сутки
+Цена в объявлении — 900 ₽/сутки при аренде от 8 суток.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
+Расходные материалы оплачиваются отдельно.
 Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
       </x:c>
       <x:c r="G10" s="8" t="str">
@@ -1699,7 +1697,7 @@
         <x:v>Строительное оборудование</x:v>
       </x:c>
       <x:c r="K10" s="10" t="n">
-        <x:v>1200</x:v>
+        <x:v>900</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="285" customHeight="1">
@@ -1723,7 +1721,9 @@
 1–3 суток — 1 100 ₽/сутки
 4–7 суток — 900 ₽/сутки
 от 8 суток — 800 ₽/сутки
+Цена в объявлении — 800 ₽/сутки при аренде от 8 суток.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
+Расходные материалы оплачиваются отдельно.
 Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
       </x:c>
       <x:c r="G11" s="8" t="str">
@@ -1739,7 +1739,7 @@
         <x:v>Строительное оборудование</x:v>
       </x:c>
       <x:c r="K11" s="10" t="n">
-        <x:v>1100</x:v>
+        <x:v>800</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="285" customHeight="1">
@@ -1763,7 +1763,9 @@
 1 сутки — 1 300 ₽/сутки
 2–7 суток — 1 100 ₽/сутки
 от 8 суток — 1 050 ₽/сутки
+Цена в объявлении — 1 050 ₽/сутки при аренде от 8 суток.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
+Расходные материалы оплачиваются отдельно.
 Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
       </x:c>
       <x:c r="G12" s="8" t="str">
@@ -1779,7 +1781,7 @@
         <x:v>Строительное оборудование</x:v>
       </x:c>
       <x:c r="K12" s="10" t="n">
-        <x:v>1300</x:v>
+        <x:v>1050</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="285" customHeight="1">
@@ -1803,7 +1805,9 @@
 1–2 суток — 1 800 ₽/сутки
 3–6 суток — 1 550 ₽/сутки
 от 7 суток — 1 400 ₽/сутки
+Цена в объявлении — 1 400 ₽/сутки при аренде от 7 суток.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
+Расходные материалы оплачиваются отдельно.
 Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
       </x:c>
       <x:c r="G13" s="8" t="str">
@@ -1819,7 +1823,7 @@
         <x:v>Строительное оборудование</x:v>
       </x:c>
       <x:c r="K13" s="10" t="n">
-        <x:v>1800</x:v>
+        <x:v>1400</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="285" customHeight="1">
@@ -1843,7 +1847,9 @@
 1–2 суток — 1 100 ₽/сутки
 3–7 суток — 1 000 ₽/сутки
 от 8 суток — 950 ₽/сутки
+Цена в объявлении — 950 ₽/сутки при аренде от 8 суток.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
+Расходные материалы оплачиваются отдельно.
 Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
       </x:c>
       <x:c r="G14" s="8" t="str">
@@ -1859,7 +1865,7 @@
         <x:v>Строительное оборудование</x:v>
       </x:c>
       <x:c r="K14" s="10" t="n">
-        <x:v>1100</x:v>
+        <x:v>950</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="285" customHeight="1">
@@ -1883,7 +1889,9 @@
 1–3 суток — 950 ₽/сутки
 4–7 суток — 800 ₽/сутки
 от 8 суток — 750 ₽/сутки
+Цена в объявлении — 750 ₽/сутки при аренде от 8 суток.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
+Расходные материалы оплачиваются отдельно.
 Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
       </x:c>
       <x:c r="G15" s="8" t="str">
@@ -1899,7 +1907,7 @@
         <x:v>Строительное оборудование</x:v>
       </x:c>
       <x:c r="K15" s="10" t="n">
-        <x:v>950</x:v>
+        <x:v>750</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="285" customHeight="1">
@@ -1923,7 +1931,9 @@
 1–2 суток — 1 050 ₽/сутки
 3–6 суток — 850 ₽/сутки
 от 7 суток — 750 ₽/сутки
+Цена в объявлении — 750 ₽/сутки при аренде от 7 суток.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
+Расходные материалы оплачиваются отдельно.
 Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
       </x:c>
       <x:c r="G16" s="8" t="str">
@@ -1939,7 +1949,7 @@
         <x:v>Строительное оборудование</x:v>
       </x:c>
       <x:c r="K16" s="10" t="n">
-        <x:v>1050</x:v>
+        <x:v>750</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="285" customHeight="1">
@@ -1963,7 +1973,9 @@
 1–3 суток — 650 ₽/сутки
 4–7 суток — 600 ₽/сутки
 от 8 суток — 550 ₽/сутки
+Цена в объявлении — 550 ₽/сутки при аренде от 8 суток.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
+Расходные материалы оплачиваются отдельно.
 Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
       </x:c>
       <x:c r="G17" s="8" t="str">
@@ -1979,7 +1991,7 @@
         <x:v>Строительное оборудование</x:v>
       </x:c>
       <x:c r="K17" s="10" t="n">
-        <x:v>650</x:v>
+        <x:v>550</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="285" customHeight="1">
@@ -2003,7 +2015,9 @@
 1–3 суток — 330 ₽/сутки
 4–7 суток — 270 ₽/сутки
 от 8 суток — 240 ₽/сутки
+Цена в объявлении — 240 ₽/сутки при аренде от 8 суток.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
+Расходные материалы оплачиваются отдельно.
 Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
       </x:c>
       <x:c r="G18" s="8" t="str">
@@ -2019,7 +2033,7 @@
         <x:v>Строительное оборудование</x:v>
       </x:c>
       <x:c r="K18" s="10" t="n">
-        <x:v>330</x:v>
+        <x:v>240</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="285" customHeight="1">
@@ -2043,7 +2057,9 @@
 1–3 суток — 650 ₽/сутки
 4–7 суток — 550 ₽/сутки
 от 8 суток — 500 ₽/сутки
+Цена в объявлении — 500 ₽/сутки при аренде от 8 суток.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
+Расходные материалы оплачиваются отдельно.
 Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
       </x:c>
       <x:c r="G19" s="8" t="str">
@@ -2059,7 +2075,7 @@
         <x:v>Строительное оборудование</x:v>
       </x:c>
       <x:c r="K19" s="10" t="n">
-        <x:v>650</x:v>
+        <x:v>500</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="285" customHeight="1">
@@ -2083,7 +2099,9 @@
 1–3 суток — 700 ₽/сутки
 4–7 суток — 650 ₽/сутки
 от 8 суток — 600 ₽/сутки
+Цена в объявлении — 600 ₽/сутки при аренде от 8 суток.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
+Расходные материалы оплачиваются отдельно.
 Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
       </x:c>
       <x:c r="G20" s="8" t="str">
@@ -2099,7 +2117,7 @@
         <x:v>Строительное оборудование</x:v>
       </x:c>
       <x:c r="K20" s="10" t="n">
-        <x:v>700</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="285" customHeight="1">
@@ -2123,7 +2141,9 @@
 1–2 суток — 550 ₽/сутки
 3–7 суток — 500 ₽/сутки
 от 8 суток — 450 ₽/сутки
+Цена в объявлении — 450 ₽/сутки при аренде от 8 суток.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
+Расходные материалы оплачиваются отдельно.
 Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
       </x:c>
       <x:c r="G21" s="8" t="str">
@@ -2139,7 +2159,7 @@
         <x:v>Строительное оборудование</x:v>
       </x:c>
       <x:c r="K21" s="10" t="n">
-        <x:v>550</x:v>
+        <x:v>450</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="285" customHeight="1">
@@ -2160,11 +2180,13 @@
         <x:v>Прокат бензореза CHAMPION CP350 в Калининграде и области. Бензорез мощностью 3,5 кВт (4,8 л.с.) для резки бетона, асфальта, камня и металла с подходящим диском. Диаметр диска — 350 мм, глубина реза — до 125 мм. Предусмотрена подача воды для мокрой резки. Диск под материал, условия оплаты его износа и топливо согласуем при оформлении аренды.
 Характеристики: мощность — 3,5 кВт / 4,8 л.с.; диаметр диска — 350 мм; глубина реза — до 125 мм; резка — сухая и мокрая с подходящим диском.
 Стоимость аренды за сутки:
-1–2 суток — 2 150 ₽/сутки
-3–7 суток — 2 000 ₽/сутки
-от 8 суток — 1 900 ₽/сутки
+1–2 суток — 2 250 ₽/сутки
+3–7 суток — 2 100 ₽/сутки
+от 8 суток — 2 000 ₽/сутки
+Цена в объявлении — 2 000 ₽/сутки при аренде от 8 суток.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Топливо в стоимость аренды не входит.
+Расходные материалы оплачиваются отдельно.
 Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
       </x:c>
       <x:c r="G22" s="8" t="str">
@@ -2180,7 +2202,7 @@
         <x:v>Строительное оборудование</x:v>
       </x:c>
       <x:c r="K22" s="10" t="n">
-        <x:v>2150</x:v>
+        <x:v>2000</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="285" customHeight="1">
@@ -2204,7 +2226,9 @@
 1–3 суток — 1 400 ₽/сутки
 4–7 суток — 1 100 ₽/сутки
 от 8 суток — 1 000 ₽/сутки
+Цена в объявлении — 1 000 ₽/сутки при аренде от 8 суток.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
+Расходные материалы оплачиваются отдельно.
 Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
       </x:c>
       <x:c r="G23" s="8" t="str">
@@ -2220,7 +2244,7 @@
         <x:v>Строительное оборудование</x:v>
       </x:c>
       <x:c r="K23" s="10" t="n">
-        <x:v>1400</x:v>
+        <x:v>1000</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2239,10 +2263,10 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="Read61ea7a07a4477"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="R57975cd0082743aa"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="R3a7f3d851f8b4003"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="Rd1f08e4287554ec5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="Re77edada2ac846f9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="R91b4b89abeb74908"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="Rfe9478ebfc1142d0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="Ra371ec1381d34c1e"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2267,16 +2291,16 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="H2" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="I2" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="H2" t="s">
+      <x:c r="J2" t="s">
         <x:v>55</x:v>
-      </x:c>
-      <x:c r="I2" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="J2" t="s">
-        <x:v>57</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Improve Avito titles and descriptions for 19 rental listings
</commit_message>
<xml_diff>
--- a/stroyrent39-avito-19-2026-09-30.xlsx
+++ b/stroyrent39-avito-19-2026-09-30.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" r:id="Rc94d02b866344408"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объявления" sheetId="2" r:id="Rbc3b52e0403640de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Справочники" sheetId="3" r:id="Rab715bfd40364489"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" r:id="R1f24661563524d44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объявления" sheetId="2" r:id="R1e7175e26efd4a64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Справочники" sheetId="3" r:id="Rbab9ba776d6c49bc"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="Instructions" localSheetId="0">Инструкция!$1:$50</x:definedName>
@@ -1303,13 +1303,13 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="Rdf2c534d021a4a85"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="Re48645af10114a50"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="Rb97e80e103514a53"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="R514e0e2dd4f64d51"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="R47afc86d016e4553"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="R675692cdb59d41a2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="Rd44b8462277e4be5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="R808fc13cc9d142ac"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="R96d134f524ef41ff"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="R4f8f97d99d7948aa"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="R803c177649fc417c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="Re3215fd82eab4664"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="R544d17aaa2ae4d4f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="Rf3b362cb760946db"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1455,20 +1455,19 @@
         <x:v>sr39-fubag-bs-9000-a-es</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>Аренда бензогенератора FUBAG BS 9000, 8,5 кВт</x:v>
+        <x:v>Аренда бензогенератора FUBAG BS 9000 A ES 8,5 кВт</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>Прокат бензогенератора FUBAG BS 9000 A ES в Калининграде и области. Бензиновый генератор мощностью 8,5 кВт для инструмента и освещения на объекте. Электростартер упрощает запуск, цифровой дисплей помогает контролировать работу.
-Характеристики: номинальная мощность — 8,5 кВт; напряжение — 220 В; запуск — электростартер; топливный бак — 36 л.
+        <x:v>Аренда бензогенератора FUBAG BS 9000 A ES в Калининграде для временного питания электроинструмента и освещения на объекте.
+Цена в объявлении — 1 600 ₽/сутки при аренде от 8 суток.
+Номинальная мощность электростанции — 8,5 кВт, напряжение 220 В. Электростартер, цифровой дисплей, бак 36 л; две розетки 16 А и одна 32 А.
 Стоимость аренды за сутки:
 1–3 суток — 2 100 ₽/сутки
 4–7 суток — 1 650 ₽/сутки
 от 8 суток — 1 600 ₽/сутки
-Цена в объявлении — 1 600 ₽/сутки при аренде от 8 суток.
+Топливо и другие расходные материалы оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
-Топливо в стоимость аренды не входит.
-Расходные материалы оплачиваются отдельно.
-Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
+Напишите в чат Авито даты аренды и суммарную мощность приборов — проверим доступность и подскажем по нагрузке.</x:v>
       </x:c>
       <x:c r="G5" s="8" t="str">
         <x:v>Калининград</x:v>
@@ -1498,20 +1497,19 @@
         <x:v>sr39-fubag-bs-6600-a-es</x:v>
       </x:c>
       <x:c r="E6" s="9" t="str">
-        <x:v>Аренда бензогенератора FUBAG BS 6600, 6 кВт</x:v>
+        <x:v>Аренда бензогенератора FUBAG BS 6600 A ES 6 кВт</x:v>
       </x:c>
       <x:c r="F6" s="9" t="str">
-        <x:v>Прокат бензогенератора FUBAG BS 6600 A ES в Калининграде и области. Бензиновый генератор мощностью 6 кВт для инструмента и освещения на объекте. Электростартер упрощает запуск, цифровой дисплей помогает контролировать работу.
-Характеристики: номинальная мощность — 6 кВт; напряжение — 220 В; запуск — электростартер; топливный бак — 25 л.
+        <x:v>Бензогенератор FUBAG BS 6600 A ES в аренду в Калининграде для временного электроснабжения инструмента и света на объекте.
+Цена в объявлении — 1 250 ₽/сутки при аренде от 8 суток.
+Номинальная мощность — 6 кВт, сеть 220 В. Есть электростартер и цифровой дисплей; бак 25 л, две розетки 16 А и одна 32 А.
 Стоимость аренды за сутки:
 1–2 суток — 1 800 ₽/сутки
 3–7 суток — 1 300 ₽/сутки
 от 8 суток — 1 250 ₽/сутки
-Цена в объявлении — 1 250 ₽/сутки при аренде от 8 суток.
+Топливо и другие расходные материалы оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
-Топливо в стоимость аренды не входит.
-Расходные материалы оплачиваются отдельно.
-Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
+Напишите в чат Авито нужные даты и мощность подключаемых приборов — уточним наличие и подходящую нагрузку.</x:v>
       </x:c>
       <x:c r="G6" s="8" t="str">
         <x:v>Калининград</x:v>
@@ -1541,20 +1539,19 @@
         <x:v>sr39-fubag-bs-3300-a-es</x:v>
       </x:c>
       <x:c r="E7" s="9" t="str">
-        <x:v>Аренда бензогенератора FUBAG BS 3300, 3 кВт</x:v>
+        <x:v>Аренда бензогенератора FUBAG BS 3300 A ES 3 кВт</x:v>
       </x:c>
       <x:c r="F7" s="9" t="str">
-        <x:v>Прокат бензогенератора FUBAG BS 3300 A ES в Калининграде и области. Бензиновый генератор мощностью 3 кВт для инструмента и освещения на объекте. Электростартер упрощает запуск, цифровой дисплей помогает контролировать работу.
-Характеристики: номинальная мощность — 3 кВт; напряжение — 220 В; запуск — электростартер; топливный бак — 15 л.
+        <x:v>Прокат бензинового генератора FUBAG BS 3300 A ES в Калининграде для питания инструмента и освещения там, где нет сети.
+Цена в объявлении — 950 ₽/сутки при аренде от 8 суток.
+Номинальная мощность — 3 кВт при 220 В. Электростартер, цифровой дисплей, бак 15 л и две розетки 16 А; параметры нагрузки согласуем до выдачи.
 Стоимость аренды за сутки:
 1–3 суток — 1 300 ₽/сутки
 4–7 суток — 1 050 ₽/сутки
 от 8 суток — 950 ₽/сутки
-Цена в объявлении — 950 ₽/сутки при аренде от 8 суток.
+Топливо и другие расходные материалы оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
-Топливо в стоимость аренды не входит.
-Расходные материалы оплачиваются отдельно.
-Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
+Укажите в сообщении Авито даты и какие приборы планируете подключать — проверим доступность генератора.</x:v>
       </x:c>
       <x:c r="G7" s="8" t="str">
         <x:v>Калининград</x:v>
@@ -1587,17 +1584,16 @@
         <x:v>Аренда виброплиты CHAMPION PC1151FT, 103 кг</x:v>
       </x:c>
       <x:c r="F8" s="9" t="str">
-        <x:v>Прокат виброплиты CHAMPION PC1151FT в Калининграде и области. Бензиновая виброплита для уплотнения песка, гравия и брусчатки. Коврик для работы по плитке — бесплатно в комплекте с арендой.
-Характеристики: центробежная сила — 25 кН; размер плиты — 500 × 580 мм; глубина уплотнения — 350 мм; вес — 103,4 кг.
+        <x:v>Аренда бензиновой виброплиты CHAMPION PC1151FT в Калининграде для уплотнения песка, гравия и основания под брусчатку.
+Цена в объявлении — 1 900 ₽/сутки при аренде от 8 суток.
+Вес 103,4 кг, центробежная сила 25 кН, плита 500 × 580 мм, глубина уплотнения до 350 мм. Коврик для плитки входит в аренду бесплатно; есть транспортировочные колёса.
 Стоимость аренды за сутки:
 1–2 суток — 2 200 ₽/сутки
 3–7 суток — 2 000 ₽/сутки
 от 8 суток — 1 900 ₽/сутки
-Цена в объявлении — 1 900 ₽/сутки при аренде от 8 суток.
+Топливо и другие расходные материалы оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
-Топливо в стоимость аренды не входит.
-Расходные материалы оплачиваются отдельно.
-Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
+Напишите в чат Авито даты и тип покрытия — уточним доступность виброплиты и комплектацию.</x:v>
       </x:c>
       <x:c r="G8" s="8" t="str">
         <x:v>Калининград</x:v>
@@ -1630,17 +1626,16 @@
         <x:v>Аренда реверсивной виброплиты CHAMPION PC1645RH</x:v>
       </x:c>
       <x:c r="F9" s="9" t="str">
-        <x:v>Прокат реверсивной виброплиты CHAMPION PC1645RH в Калининграде и области. Реверсивная бензиновая виброплита для уплотнения песка, гравия и брусчатки. Обратный ход упрощает маневрирование. Коврик для работы по плитке — бесплатно в комплекте с арендой.
-Характеристики: центробежная сила — 30,5 кН; размер плиты — 730 × 450 мм; глубина уплотнения — 500 мм; вес — 152 кг.
+        <x:v>Реверсивная виброплита CHAMPION PC1645RH в аренду в Калининграде для уплотнения песка, гравия и подготовки основания под брусчатку.
+Цена в объявлении — 2 150 ₽/сутки при аренде от 8 суток.
+Вес 152 кг, усилие 30,5 кН, плита 730 × 450 мм, глубина уплотнения до 500 мм. Обратный ход помогает маневрировать; коврик для плитки входит в аренду бесплатно.
 Стоимость аренды за сутки:
 1 сутки — 2 500 ₽/сутки
 2–7 суток — 2 200 ₽/сутки
 от 8 суток — 2 150 ₽/сутки
-Цена в объявлении — 2 150 ₽/сутки при аренде от 8 суток.
+Топливо и другие расходные материалы оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
-Топливо в стоимость аренды не входит.
-Расходные материалы оплачиваются отдельно.
-Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
+Напишите в чат Авито сроки и материал основания — проверим наличие реверсивной плиты.</x:v>
       </x:c>
       <x:c r="G9" s="8" t="str">
         <x:v>Калининград</x:v>
@@ -1670,19 +1665,19 @@
         <x:v>sr39-dorn-pro-dpvc-40stc</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
-        <x:v>Аренда строительного пылесоса DORN PRO, 40 л</x:v>
+        <x:v>Аренда строительного пылесоса DORN PRO DPVC-40STC</x:v>
       </x:c>
       <x:c r="F10" s="9" t="str">
-        <x:v>Прокат строительного пылесоса DORN PRO DPVC-40STC в Калининграде и области. Строительный пылесос 1 600 Вт с баком 40 л для сухой и влажной уборки. Есть розетка для электроинструмента и автоматическая очистка фильтра. Обычная уборка: мешок не включён. Штробление и шлифовка: расход мешка оплачивается отдельно.
-Характеристики: мощность — 1 600 Вт; объём бака — 40 л; розетка для инструмента — до 2 000 Вт; тип уборки — сухая и влажная.
+        <x:v>Аренда строительного пылесоса DORN PRO DPVC-40STC в Калининграде для сухой и влажной уборки после строительных работ.
+Цена в объявлении — 900 ₽/сутки при аренде от 8 суток.
+Мощность 1 600 Вт, бак 40 л, фильтр HEPA и автоматическая очистка фильтра. Есть розетка для инструмента до 2 000 Вт и шланг 4 м — удобно при шлифовке и штроблении.
 Стоимость аренды за сутки:
 1–2 суток — 1 200 ₽/сутки
 3–7 суток — 1 000 ₽/сутки
 от 8 суток — 900 ₽/сутки
-Цена в объявлении — 900 ₽/сутки при аренде от 8 суток.
+Мешок для обычной уборки не включён. При штроблении и шлифовке расход мешка оплачивается отдельно; остальные расходные материалы тоже оплачиваются отдельно, если потребуются.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
-Расходные материалы оплачиваются отдельно.
-Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
+Напишите в чат Авито даты и тип уборки — проверим доступность пылесоса и уточним расход мешков.</x:v>
       </x:c>
       <x:c r="G10" s="8" t="str">
         <x:v>Калининград</x:v>
@@ -1715,16 +1710,16 @@
         <x:v>Аренда перфоратора Makita HR3011FCJ SDS-Plus</x:v>
       </x:c>
       <x:c r="F11" s="9" t="str">
-        <x:v>Прокат перфоратора Makita HR3011FCJ в Калининграде и области. Сетевой перфоратор SDS-Plus мощностью 1 050 Вт с энергией удара 3,9 Дж. Для сверления, сверления с ударом и долбления. Система AVT снижает вибрацию, подсветка помогает работать в слабо освещённых местах.
-Характеристики: мощность — 1 050 Вт; энергия удара — 3,9 Дж; патрон — SDS-Plus; сверление в бетоне — до 30 мм.
+        <x:v>Перфоратор Makita HR3011FCJ SDS-Plus в аренду в Калининграде для сверления дерева и металла, ударного сверления бетона и долбления.
+Цена в объявлении — 800 ₽/сутки при аренде от 8 суток.
+Мощность 1 050 Вт, удар 3,9 Дж, сверление бетона до 30 мм. AVT снижает вибрацию, подсветка помогает при слабом освещении; боковая рукоятка, ограничитель глубины и кейс в комплекте.
 Стоимость аренды за сутки:
 1–3 суток — 1 100 ₽/сутки
 4–7 суток — 900 ₽/сутки
 от 8 суток — 800 ₽/сутки
-Цена в объявлении — 800 ₽/сутки при аренде от 8 суток.
+Буры, коронки и другие расходные материалы, если понадобятся, оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
-Расходные материалы оплачиваются отдельно.
-Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
+Укажите в сообщении Авито даты, материал и диаметр отверстий — проверим наличие перфоратора.</x:v>
       </x:c>
       <x:c r="G11" s="8" t="str">
         <x:v>Калининград</x:v>
@@ -1754,19 +1749,19 @@
         <x:v>sr39-makita-hm1203c</x:v>
       </x:c>
       <x:c r="E12" s="9" t="str">
-        <x:v>Аренда отбойного молотка Makita HM1203C</x:v>
+        <x:v>Аренда отбойного молотка Makita HM1203C 19,1 Дж</x:v>
       </x:c>
       <x:c r="F12" s="9" t="str">
-        <x:v>Прокат отбойного молотка Makita HM1203C в Калининграде и области. Сетевой отбойный молоток для демонтажа бетона, кирпича и камня. Удар 19,1 Дж, патрон SDS-Max и регулировка частоты ударов для работы с разными материалами.
-Характеристики: энергия удара — 19,1 Дж; мощность — 1 510 Вт; тип патрона — SDS-Max; частота ударов — 950–1 900 уд/мин.
+        <x:v>Аренда отбойного молотка Makita HM1203C в Калининграде для демонтажа бетона, кирпича и камня.
+Цена в объявлении — 1 050 ₽/сутки при аренде от 8 суток.
+Сетевой инструмент 1 510 Вт с ударом 19,1 Дж и патроном SDS-Max. Частоту ударов можно регулировать от 950 до 1 900 в минуту; долото ставится в 12 положениях.
 Стоимость аренды за сутки:
 1 сутки — 1 300 ₽/сутки
 2–7 суток — 1 100 ₽/сутки
 от 8 суток — 1 050 ₽/сутки
-Цена в объявлении — 1 050 ₽/сутки при аренде от 8 суток.
+Расходные материалы для работ, если потребуются, оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
-Расходные материалы оплачиваются отдельно.
-Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
+Напишите в чат Авито даты и что нужно демонтировать — уточним доступность и комплектацию.</x:v>
       </x:c>
       <x:c r="G12" s="8" t="str">
         <x:v>Калининград</x:v>
@@ -1796,19 +1791,19 @@
         <x:v>sr39-foxweld-aeromax-480-100</x:v>
       </x:c>
       <x:c r="E13" s="9" t="str">
-        <x:v>Аренда компрессора FoxWeld AEROMAX 480/100</x:v>
+        <x:v>Аренда компрессора FoxWeld AEROMAX 480/100, 100 л</x:v>
       </x:c>
       <x:c r="F13" s="9" t="str">
-        <x:v>Прокат компрессора FoxWeld AEROMAX 480/100 в Калининграде и области. Масляный компрессор с ресивером 100 л для работы с пневмоинструментом. Производительность 480 л/мин, давление до 8 бар. Работает от сети 220 В, оснащён регулятором давления и защитой от перегрева.
-Характеристики: объём ресивера — 100 л; производительность — 480 л/мин; максимальное давление — 8 бар; напряжение — 220 В.
+        <x:v>Воздушный компрессор FoxWeld AEROMAX 480/100 в аренду в Калининграде для работы с пневмоинструментом.
+Цена в объявлении — 1 400 ₽/сутки при аренде от 7 суток.
+Ресивер 100 л, производительность 480 л/мин, давление до 8 бар. Масляный ременной компрессор работает от 220 В; есть регулировка давления и защита от перегрева.
 Стоимость аренды за сутки:
 1–2 суток — 1 800 ₽/сутки
 3–6 суток — 1 550 ₽/сутки
 от 7 суток — 1 400 ₽/сутки
-Цена в объявлении — 1 400 ₽/сутки при аренде от 7 суток.
+Расходные материалы для работ, если потребуются, оплачиваются отдельно; состав комплекта согласуем до выдачи.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
-Расходные материалы оплачиваются отдельно.
-Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
+Напишите в чат Авито даты и какой пневмоинструмент хотите подключить — проверим наличие и совместимость.</x:v>
       </x:c>
       <x:c r="G13" s="8" t="str">
         <x:v>Калининград</x:v>
@@ -1841,16 +1836,16 @@
         <x:v>Аренда шлифмашины для стен DORN PRO DPDS-750</x:v>
       </x:c>
       <x:c r="F14" s="9" t="str">
-        <x:v>Прокат шлифмашины для стен и потолков DORN PRO DPDS-750 в Калининграде и области. Шлифмашина для стен и потолков из гипсокартона и оштукатуренных поверхностей. Мощность 750 Вт, диск 225 мм, регулировка оборотов и подключение к пылесосу. Абразивы клиент покупает отдельно.
-Характеристики: мощность — 750 Вт; диаметр диска — 225 мм; частота вращения — 600–1 850 об/мин; подключение к пылесосу — есть.
+        <x:v>Аренда шлифмашины для стен и потолков DORN PRO DPDS-750 («жираф») в Калининграде для гипсокартона и оштукатуренных поверхностей.
+Цена в объявлении — 950 ₽/сутки при аренде от 8 суток.
+Диск 225 мм, мощность 750 Вт, регулировка 600–1 850 об/мин. Есть подсветка зоны работы и подключение к пылесосу для отвода пыли.
 Стоимость аренды за сутки:
 1–2 суток — 1 100 ₽/сутки
 3–7 суток — 1 000 ₽/сутки
 от 8 суток — 950 ₽/сутки
-Цена в объявлении — 950 ₽/сутки при аренде от 8 суток.
+Шлифлисты (абразивы) и другие расходные материалы оплачиваются отдельно. Необходимость пылесоса уточним при оформлении.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
-Расходные материалы оплачиваются отдельно.
-Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
+Укажите в сообщении Авито даты и площадь шлифовки — проверим доступность машины и подходящие абразивы.</x:v>
       </x:c>
       <x:c r="G14" s="8" t="str">
         <x:v>Калининград</x:v>
@@ -1883,16 +1878,16 @@
         <x:v>Аренда фекального насоса Oasis F-1500/13R</x:v>
       </x:c>
       <x:c r="F15" s="9" t="str">
-        <x:v>Прокат фекального насоса Oasis F-1500/13R в Калининграде и области. Погружной насос с измельчителем для откачки грязной воды и канализационных/фекальных стоков. В комплекте: два рукава по 20 м диаметром 2″, хомуты, соединители и трос. Для грязной воды — обычный тариф. Для канализационных и фекальных стоков — дополнительно 1 000 ₽ за санитарную очистку. Если очищаете оборудование самостоятельно перед возвратом, доплаты нет.
-Характеристики: мощность — 1 500 Вт; производительность — до 24 900 л/ч; максимальный напор — 13 м; измельчитель — есть.
+        <x:v>Аренда погружного фекального насоса Oasis F-1500/13R с измельчителем в Калининграде для откачки грязной воды и канализационных стоков.
+Цена в объявлении — 750 ₽/сутки при аренде от 8 суток.
+Мощность 1 500 Вт, производительность до 24 900 л/ч, напор до 13 м. В комплекте два рукава по 20 м диаметром 2″, хомуты, соединители и трос.
 Стоимость аренды за сутки:
 1–3 суток — 950 ₽/сутки
 4–7 суток — 800 ₽/сутки
 от 8 суток — 750 ₽/сутки
-Цена в объявлении — 750 ₽/сутки при аренде от 8 суток.
+Для канализационных и фекальных стоков санитарная очистка стоит дополнительно 1 000 ₽. Если очистите насос перед возвратом самостоятельно, этой доплаты нет. Расходные материалы для работ, если понадобятся, оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
-Расходные материалы оплачиваются отдельно.
-Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
+Напишите в чат Авито, что нужно откачать, глубину и даты — уточним доступность насоса и условия очистки.</x:v>
       </x:c>
       <x:c r="G15" s="8" t="str">
         <x:v>Калининград</x:v>
@@ -1925,16 +1920,16 @@
         <x:v>Аренда бетономешалки ПРОФМАШ Б180, 160 л</x:v>
       </x:c>
       <x:c r="F16" s="9" t="str">
-        <x:v>Прокат бетономешалки ПРОФМАШ Б180 в Калининграде и области. Электрическая бетономешалка с баком 160 л для приготовления бетона, кладочных и штукатурных растворов. Объём готовой смеси — 90 л. Возврат очищенной бетономешалки. Очистка при возврате с застывшим раствором — 1 500 ₽.
-Характеристики: объём бака — 160 л; объём готовой смеси — 90 л; мощность — 700 Вт; напряжение — 220 В.
+        <x:v>Бетономешалка ПРОФМАШ Б180 в аренду в Калининграде для приготовления бетона, кладочного или штукатурного раствора.
+Цена в объявлении — 750 ₽/сутки при аренде от 7 суток.
+Объём бака 160 л, готовой смеси — до 90 л; мощность 700 Вт, питание 220 В. Чугунный венец и транспортировочные колёса.
 Стоимость аренды за сутки:
 1–2 суток — 1 050 ₽/сутки
 3–6 суток — 850 ₽/сутки
 от 7 суток — 750 ₽/сутки
-Цена в объявлении — 750 ₽/сутки при аренде от 7 суток.
+Верните бетоносмеситель очищенным. Очистка при возврате с застывшим раствором стоит 1 500 ₽; расходные материалы для работ оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
-Расходные материалы оплачиваются отдельно.
-Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
+Напишите в чат Авито даты и объём работ — проверим доступность бетономешалки.</x:v>
       </x:c>
       <x:c r="G16" s="8" t="str">
         <x:v>Калининград</x:v>
@@ -1964,19 +1959,19 @@
         <x:v>sr39-ballu-bdi-50l</x:v>
       </x:c>
       <x:c r="E17" s="9" t="str">
-        <x:v>Аренда осушителя воздуха BALLU BDI-50L</x:v>
+        <x:v>Аренда осушителя BALLU BDI-50L, 50 л/сутки</x:v>
       </x:c>
       <x:c r="F17" s="9" t="str">
-        <x:v>Прокат осушителя воздуха BALLU BDI-50L в Калининграде и области. Промышленный осушитель воздуха для сушки помещений и поверхностей после строительных работ. Удаляет до 50 л влаги в сутки; фактическая производительность зависит от температуры и влажности. Встроенные гигрометр и гигростат помогают контролировать влажность.
-Характеристики: осушение — до 50 л/сутки; воздухообмен — 350 м³/ч; бак для конденсата — 7 л; гигрометр и гигростат — встроенные.
+        <x:v>Аренда промышленного осушителя воздуха BALLU BDI-50L в Калининграде для сушки помещений после ремонта и строительных работ.
+Цена в объявлении — 550 ₽/сутки при аренде от 8 суток.
+Осушение до 50 л/сутки зависит от температуры и влажности. Воздухообмен 350 м³/ч, бак 7 л; встроенные гигрометр и гигростат помогают контролировать влажность.
 Стоимость аренды за сутки:
 1–3 суток — 650 ₽/сутки
 4–7 суток — 600 ₽/сутки
 от 8 суток — 550 ₽/сутки
-Цена в объявлении — 550 ₽/сутки при аренде от 8 суток.
+Расходные материалы для ваших работ, если потребуются, оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
-Расходные материалы оплачиваются отдельно.
-Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
+Укажите в сообщении Авито площадь помещения, условия влажности и даты — проверим доступность осушителя.</x:v>
       </x:c>
       <x:c r="G17" s="8" t="str">
         <x:v>Калининград</x:v>
@@ -2006,19 +2001,19 @@
         <x:v>sr39-dorn-pro-115594</x:v>
       </x:c>
       <x:c r="E18" s="9" t="str">
-        <x:v>Аренда стремянки DORN PRO, 4 ступени</x:v>
+        <x:v>Аренда стремянки DORN PRO 115594, 4 ступени</x:v>
       </x:c>
       <x:c r="F18" s="9" t="str">
-        <x:v>Прокат стремянки DORN PRO 115594 на 4 ступени в Калининграде и области. Ультратонкая алюминиевая стремянка для ремонта, монтажа и бытовых задач. Площадка на высоте 0,91 м, ребристые ступени и поручень. В сложенном виде толщина — 55 мм: удобно перевозить и хранить.
-Характеристики: количество ступеней — 4; высота площадки — 0,91 м; максимальная нагрузка — 150 кг; вес — 6,4 кг.
+        <x:v>Аренда алюминиевой стремянки DORN PRO 115594 на 4 ступени в Калининграде для ремонта, монтажа и работ внутри помещения.
+Цена в объявлении — 240 ₽/сутки при аренде от 8 суток.
+Высота площадки 0,91 м, допустимая нагрузка до 150 кг. Ребристые ступени, поручень и противоскользящие опоры; в сложенном виде толщина всего 55 мм.
 Стоимость аренды за сутки:
 1–3 суток — 330 ₽/сутки
 4–7 суток — 270 ₽/сутки
 от 8 суток — 240 ₽/сутки
-Цена в объявлении — 240 ₽/сутки при аренде от 8 суток.
+Расходные материалы для ваших работ, если потребуются, оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
-Расходные материалы оплачиваются отдельно.
-Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
+Напишите в чат Авито нужную высоту и даты — проверим доступность стремянки.</x:v>
       </x:c>
       <x:c r="G18" s="8" t="str">
         <x:v>Калининград</x:v>
@@ -2048,19 +2043,19 @@
         <x:v>sr39-novaya-vysota-200-10</x:v>
       </x:c>
       <x:c r="E19" s="9" t="str">
-        <x:v>Аренда стремянки Новая Высота, 10 ступеней</x:v>
+        <x:v>Аренда стремянки Новая Высота 200, 10 ступеней</x:v>
       </x:c>
       <x:c r="F19" s="9" t="str">
-        <x:v>Прокат стремянки Новая Высота 200 на 10 ступеней в Калининграде и области. Алюминиевая стремянка серии 200 для ремонта и монтажных работ. Площадка на высоте 2,17 м, органайзер для инструмента и крюк для ведра. Рифлёные ступени и противоскользящие опоры, максимальная нагрузка — 180 кг.
-Характеристики: количество ступеней — 10; высота площадки — 2,17 м; максимальная нагрузка — 180 кг; рабочая высота по данным производителя — 4,17 м.
+        <x:v>Прокат алюминиевой стремянки Новая Высота 200 на 10 ступеней в Калининграде для ремонта и монтажных работ на высоте.
+Цена в объявлении — 500 ₽/сутки при аренде от 8 суток.
+Площадка на высоте 2,17 м, допустимая нагрузка до 180 кг. Есть органайзер для инструмента, крюк для ведра, рифлёные ступени и противоскользящие опоры.
 Стоимость аренды за сутки:
 1–3 суток — 650 ₽/сутки
 4–7 суток — 550 ₽/сутки
 от 8 суток — 500 ₽/сутки
-Цена в объявлении — 500 ₽/сутки при аренде от 8 суток.
+Расходные материалы для ваших работ, если потребуются, оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
-Расходные материалы оплачиваются отдельно.
-Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
+Укажите в сообщении Авито нужную высоту и даты — проверим доступность стремянки.</x:v>
       </x:c>
       <x:c r="G19" s="8" t="str">
         <x:v>Калининград</x:v>
@@ -2093,16 +2088,16 @@
         <x:v>Аренда шуруповёрта Makita DDF484RME, 18 В</x:v>
       </x:c>
       <x:c r="F20" s="9" t="str">
-        <x:v>Прокат шуруповёрта Makita DDF484RME в Калининграде и области. Аккумуляторный бесщёточный шуруповёрт 18 В для крепежа и сверления дерева, металла и пластика. Две скорости, быстрозажимной патрон и подсветка для работы в слабо освещённых местах. Свёрла отдельно.
-Характеристики: напряжение — 18 В; крутящий момент — 54 Н·м; аккумуляторы — 2 × 4,0 А·ч, Li-Ion; патрон — быстрозажимной, 1,5–13 мм.
+        <x:v>Аккумуляторная дрель-шуруповёрт Makita DDF484RME в аренду в Калининграде для крепежа и сверления дерева, металла и пластика.
+Цена в объявлении — 600 ₽/сутки при аренде от 8 суток.
+Бесщёточный двигатель 18 В, момент 54 Н·м, две скорости и подсветка. В комплекте два аккумулятора 4,0 А·ч, зарядное устройство и кейс; ударного режима нет.
 Стоимость аренды за сутки:
 1–3 суток — 700 ₽/сутки
 4–7 суток — 650 ₽/сутки
 от 8 суток — 600 ₽/сутки
-Цена в объявлении — 600 ₽/сутки при аренде от 8 суток.
+Свёрла и другие расходные материалы оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
-Расходные материалы оплачиваются отдельно.
-Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
+Напишите в чат Авито даты и материал для сверления — уточним доступность шуруповёрта.</x:v>
       </x:c>
       <x:c r="G20" s="8" t="str">
         <x:v>Калининград</x:v>
@@ -2135,16 +2130,16 @@
         <x:v>Аренда строительного фена Makita HG5030K</x:v>
       </x:c>
       <x:c r="F21" s="9" t="str">
-        <x:v>Прокат строительного фена Makita HG5030K в Калининграде и области. Технический фен мощностью 1 600 Вт для сушки и размягчения материалов. Два режима нагрева: 350 и 500 °C. Нескользящая рукоятка для удобного хвата, плоская задняя часть для стационарной установки.
-Характеристики: мощность — 1 600 Вт; рабочая температура — 350 / 500 °C; воздушный поток — 300 / 500 л/мин; количество режимов — 2.
+        <x:v>Аренда строительного фена Makita HG5030K в Калининграде для сушки и размягчения материалов при ремонте.
+Цена в объявлении — 450 ₽/сутки при аренде от 8 суток.
+Технический фен 1 600 Вт с режимами 350 и 500 °C, потоком воздуха 300 и 500 л/мин. В комплекте четыре насадки и кейс; возможна стационарная установка.
 Стоимость аренды за сутки:
 1–2 суток — 550 ₽/сутки
 3–7 суток — 500 ₽/сутки
 от 8 суток — 450 ₽/сутки
-Цена в объявлении — 450 ₽/сутки при аренде от 8 суток.
+Расходные материалы для ваших работ, если потребуются, оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
-Расходные материалы оплачиваются отдельно.
-Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
+Укажите в сообщении Авито материал, задачу и даты — проверим доступность термофена.</x:v>
       </x:c>
       <x:c r="G21" s="8" t="str">
         <x:v>Калининград</x:v>
@@ -2177,17 +2172,16 @@
         <x:v>Аренда бензореза CHAMPION CP350, диск 350 мм</x:v>
       </x:c>
       <x:c r="F22" s="9" t="str">
-        <x:v>Прокат бензореза CHAMPION CP350 в Калининграде и области. Бензорез мощностью 3,5 кВт (4,8 л.с.) для резки бетона, асфальта, камня и металла с подходящим диском. Диаметр диска — 350 мм, глубина реза — до 125 мм. Предусмотрена подача воды для мокрой резки. Диск под материал, условия оплаты его износа и топливо согласуем при оформлении аренды.
-Характеристики: мощность — 3,5 кВт / 4,8 л.с.; диаметр диска — 350 мм; глубина реза — до 125 мм; резка — сухая и мокрая с подходящим диском.
+        <x:v>Бензорез CHAMPION CP350 в аренду в Калининграде для резки бетона, асфальта и камня; металл режется с подходящим диском.
+Цена в объявлении — 2 000 ₽/сутки при аренде от 8 суток.
+Мощность 3,5 кВт, диск 350 мм, глубина реза до 125 мм. Возможна сухая и мокрая резка с подходящим диском; предусмотрена подача воды.
 Стоимость аренды за сутки:
 1–2 суток — 2 250 ₽/сутки
 3–7 суток — 2 100 ₽/сутки
 от 8 суток — 2 000 ₽/сутки
-Цена в объявлении — 2 000 ₽/сутки при аренде от 8 суток.
+Топливо и расходные материалы оплачиваются отдельно. Диск под материал и условия оплаты его износа согласуем до выдачи.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
-Топливо в стоимость аренды не входит.
-Расходные материалы оплачиваются отдельно.
-Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
+Напишите в чат Авито материал, глубину реза и даты — уточним доступность бензореза и условия по диску.</x:v>
       </x:c>
       <x:c r="G22" s="8" t="str">
         <x:v>Калининград</x:v>
@@ -2217,19 +2211,19 @@
         <x:v>sr39-zubr-zsh-p65-2700-pstk</x:v>
       </x:c>
       <x:c r="E23" s="9" t="str">
-        <x:v>Аренда штробореза ЗУБР ЗШ-П65-2700, 230 мм</x:v>
+        <x:v>Аренда штробореза ЗУБР ЗШ-П65-2700 ПСТК</x:v>
       </x:c>
       <x:c r="F23" s="9" t="str">
-        <x:v>Прокат штробореза ЗУБР ЗШ-П65-2700 ПСТК в Калининграде и области. Штроборез мощностью 2 700 Вт для прокладки каналов в бетоне и кирпиче. Два диска диаметром 230 мм, глубина реза до 65 мм и ширина штробы до 40 мм. Плавный пуск и поддержание оборотов для работы под нагрузкой. Подбор дисков и условия оплаты их износа согласуем при оформлении аренды. Строительный пылесос арендуется отдельно.
-Характеристики: мощность — 2 700 Вт; диаметр диска — 230 мм; глубина реза — до 65 мм; ширина штробы — 4,3–40 мм.
+        <x:v>Аренда штробореза ЗУБР ЗШ-П65-2700 ПСТК в Калининграде для прокладки каналов в бетоне и кирпиче.
+Цена в объявлении — 1 000 ₽/сутки при аренде от 8 суток.
+Бороздодел 2 700 Вт работает с двумя дисками 230 мм: глубина реза до 65 мм, ширина штробы 4,3–40 мм. Есть плавный пуск и подключение к пылесосу.
 Стоимость аренды за сутки:
 1–3 суток — 1 400 ₽/сутки
 4–7 суток — 1 100 ₽/сутки
 от 8 суток — 1 000 ₽/сутки
-Цена в объявлении — 1 000 ₽/сутки при аренде от 8 суток.
+Подбор дисков и условия оплаты их износа согласуем до выдачи. Строительный пылесос арендуется отдельно; расходные материалы оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
-Расходные материалы оплачиваются отдельно.
-Напишите в сообщения Авито, чтобы уточнить свободные даты и комплектацию.</x:v>
+Напишите в чат Авито материал стены, размеры штробы и даты — проверим доступность инструмента.</x:v>
       </x:c>
       <x:c r="G23" s="8" t="str">
         <x:v>Калининград</x:v>
@@ -2263,10 +2257,10 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="Re77edada2ac846f9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="R91b4b89abeb74908"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="Rfe9478ebfc1142d0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="Ra371ec1381d34c1e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="R41f98b116d7d47f7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="R0e338bd23cda4bc1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="R3e53ed7310b64f11"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="Ra8a6a9d559aa4ad4"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Refine Avito rental titles with precise search synonyms
</commit_message>
<xml_diff>
--- a/stroyrent39-avito-19-2026-09-30.xlsx
+++ b/stroyrent39-avito-19-2026-09-30.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" r:id="R1f24661563524d44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объявления" sheetId="2" r:id="R1e7175e26efd4a64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Справочники" sheetId="3" r:id="Rbab9ba776d6c49bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" r:id="R1d1c80665f2b4f2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объявления" sheetId="2" r:id="Raa10b13ab70b4f7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Справочники" sheetId="3" r:id="R42aa7dfe58e64ab8"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="Instructions" localSheetId="0">Инструкция!$1:$50</x:definedName>
@@ -1303,13 +1303,13 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="R808fc13cc9d142ac"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="R96d134f524ef41ff"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="R4f8f97d99d7948aa"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="R803c177649fc417c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="Re3215fd82eab4664"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="R544d17aaa2ae4d4f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="Rf3b362cb760946db"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="R1f74f7401ccc4cea"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="Ra01c4eee110f42e0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="R43ee89668dc941ec"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="Rcdfc80defbb8408d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="R68be67b5d3c44e14"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="R3cd840736d034ce8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="R9841c48bb7204f4c"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1581,7 +1581,7 @@
         <x:v>sr39-champion-pc1151ft</x:v>
       </x:c>
       <x:c r="E8" s="9" t="str">
-        <x:v>Аренда виброплиты CHAMPION PC1151FT, 103 кг</x:v>
+        <x:v>Аренда виброплиты CHAMPION PC1151FT для трамбовки</x:v>
       </x:c>
       <x:c r="F8" s="9" t="str">
         <x:v>Аренда бензиновой виброплиты CHAMPION PC1151FT в Калининграде для уплотнения песка, гравия и основания под брусчатку.
@@ -1749,7 +1749,7 @@
         <x:v>sr39-makita-hm1203c</x:v>
       </x:c>
       <x:c r="E12" s="9" t="str">
-        <x:v>Аренда отбойного молотка Makita HM1203C 19,1 Дж</x:v>
+        <x:v>Аренда отбойного молотка Makita HM1203C (отбойник)</x:v>
       </x:c>
       <x:c r="F12" s="9" t="str">
         <x:v>Аренда отбойного молотка Makita HM1203C в Калининграде для демонтажа бетона, кирпича и камня.
@@ -1833,7 +1833,7 @@
         <x:v>sr39-dorn-pro-dpds-750</x:v>
       </x:c>
       <x:c r="E14" s="9" t="str">
-        <x:v>Аренда шлифмашины для стен DORN PRO DPDS-750</x:v>
+        <x:v>Аренда шлифмашины «жираф» DORN PRO DPDS-750</x:v>
       </x:c>
       <x:c r="F14" s="9" t="str">
         <x:v>Аренда шлифмашины для стен и потолков DORN PRO DPDS-750 («жираф») в Калининграде для гипсокартона и оштукатуренных поверхностей.
@@ -1959,7 +1959,7 @@
         <x:v>sr39-ballu-bdi-50l</x:v>
       </x:c>
       <x:c r="E17" s="9" t="str">
-        <x:v>Аренда осушителя BALLU BDI-50L, 50 л/сутки</x:v>
+        <x:v>Аренда осушителя воздуха BALLU BDI-50L</x:v>
       </x:c>
       <x:c r="F17" s="9" t="str">
         <x:v>Аренда промышленного осушителя воздуха BALLU BDI-50L в Калининграде для сушки помещений после ремонта и строительных работ.
@@ -2085,7 +2085,7 @@
         <x:v>sr39-makita-ddf484rme</x:v>
       </x:c>
       <x:c r="E20" s="9" t="str">
-        <x:v>Аренда шуруповёрта Makita DDF484RME, 18 В</x:v>
+        <x:v>Аренда дрели-шуруповёрта Makita DDF484RME, 18 В</x:v>
       </x:c>
       <x:c r="F20" s="9" t="str">
         <x:v>Аккумуляторная дрель-шуруповёрт Makita DDF484RME в аренду в Калининграде для крепежа и сверления дерева, металла и пластика.
@@ -2169,7 +2169,7 @@
         <x:v>sr39-champion-cp350</x:v>
       </x:c>
       <x:c r="E22" s="9" t="str">
-        <x:v>Аренда бензореза CHAMPION CP350, диск 350 мм</x:v>
+        <x:v>Аренда бензореза CHAMPION CP350 под диск 350 мм</x:v>
       </x:c>
       <x:c r="F22" s="9" t="str">
         <x:v>Бензорез CHAMPION CP350 в аренду в Калининграде для резки бетона, асфальта и камня; металл режется с подходящим диском.
@@ -2211,7 +2211,7 @@
         <x:v>sr39-zubr-zsh-p65-2700-pstk</x:v>
       </x:c>
       <x:c r="E23" s="9" t="str">
-        <x:v>Аренда штробореза ЗУБР ЗШ-П65-2700 ПСТК</x:v>
+        <x:v>Аренда штробореза ЗУБР ЗШ-П65-2700 (бороздодел)</x:v>
       </x:c>
       <x:c r="F23" s="9" t="str">
         <x:v>Аренда штробореза ЗУБР ЗШ-П65-2700 ПСТК в Калининграде для прокладки каналов в бетоне и кирпиче.
@@ -2257,10 +2257,10 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="R41f98b116d7d47f7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="R0e338bd23cda4bc1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="R3e53ed7310b64f11"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="Ra8a6a9d559aa4ad4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="R66060ec102ff4d0c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="Re827b5d903a34f56"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="R8c3380646a9c4cfd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="R7b2811513a024443"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Clarify CHAMPION CP350 diamond disc wear terms
</commit_message>
<xml_diff>
--- a/stroyrent39-avito-19-2026-09-30.xlsx
+++ b/stroyrent39-avito-19-2026-09-30.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" r:id="R1d1c80665f2b4f2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объявления" sheetId="2" r:id="Raa10b13ab70b4f7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Справочники" sheetId="3" r:id="R42aa7dfe58e64ab8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" r:id="R05eb15f64b4d4b38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объявления" sheetId="2" r:id="Rd5d1fd622df54647"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Справочники" sheetId="3" r:id="R20db4aa99331467a"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="Instructions" localSheetId="0">Инструкция!$1:$50</x:definedName>
@@ -1303,13 +1303,13 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="R1f74f7401ccc4cea"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="Ra01c4eee110f42e0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="R43ee89668dc941ec"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="Rcdfc80defbb8408d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="R68be67b5d3c44e14"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="R3cd840736d034ce8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="R9841c48bb7204f4c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="Rf19cdd008f184b70"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="Rcf07c1dd99744de8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="R82c455b015264575"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="R0af535adba1b43ea"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="R02f41cde35684a21"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="R882ab43f03164352"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="Rbbc9e78afa89455f"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2179,9 +2179,9 @@
 1–2 суток — 2 250 ₽/сутки
 3–7 суток — 2 100 ₽/сутки
 от 8 суток — 2 000 ₽/сутки
-Топливо и расходные материалы оплачиваются отдельно. Диск под материал и условия оплаты его износа согласуем до выдачи.
+Топливо и прочие расходные материалы оплачиваются отдельно. Износ нашего алмазного диска 350 мм оплачивается по факту — 1 000 ₽/мм; минимальное списание 0,5 мм = 500 ₽. При использовании своего совместимого диска доплаты за износ нет.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
-Напишите в чат Авито материал, глубину реза и даты — уточним доступность бензореза и условия по диску.</x:v>
+Напишите в чат Авито материал, глубину реза и даты. Если у вас свой диск, укажите его параметры — уточним совместимость и доступность бензореза.</x:v>
       </x:c>
       <x:c r="G22" s="8" t="str">
         <x:v>Калининград</x:v>
@@ -2257,10 +2257,10 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="R66060ec102ff4d0c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="Re827b5d903a34f56"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="R8c3380646a9c4cfd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="R7b2811513a024443"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="R507035b5d2dd43ae"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="Rcfc385d250aa44f1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="R28a0f27ed7ec49e2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="Rac306d85ae4c477c"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Update Avito XLSX feed with 2026-10-02 data
</commit_message>
<xml_diff>
--- a/stroyrent39-avito-19-2026-09-30.xlsx
+++ b/stroyrent39-avito-19-2026-09-30.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" r:id="R05eb15f64b4d4b38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объявления" sheetId="2" r:id="Rd5d1fd622df54647"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Справочники" sheetId="3" r:id="R20db4aa99331467a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" r:id="Re3953f24f6a84d98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объявления" sheetId="2" r:id="Ra4bd3f90f98046ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Справочники" sheetId="3" r:id="R1a8b3dc00730408a"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="Instructions" localSheetId="0">Инструкция!$1:$50</x:definedName>
@@ -1303,13 +1303,13 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="Rf19cdd008f184b70"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="Rcf07c1dd99744de8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="R82c455b015264575"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="R0af535adba1b43ea"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="R02f41cde35684a21"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="R882ab43f03164352"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="Rbbc9e78afa89455f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="R128ae135a3fd4456"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="R9004f87e3b364176"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="R2860d14a3a4f486e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="R3b118e96bd5e429e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="Rc2363564df274ea8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="R9a99d80364b04a27"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="R2eb6697129c946a1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1460,11 +1460,13 @@
       <x:c r="F5" s="9" t="str">
         <x:v>Аренда бензогенератора FUBAG BS 9000 A ES в Калининграде для временного питания электроинструмента и освещения на объекте.
 Цена в объявлении — 1 600 ₽/сутки при аренде от 8 суток.
+📋 Характеристики
 Номинальная мощность электростанции — 8,5 кВт, напряжение 220 В. Электростартер, цифровой дисплей, бак 36 л; две розетки 16 А и одна 32 А.
-Стоимость аренды за сутки:
+💰 Стоимость аренды за сутки:
 1–3 суток — 2 100 ₽/сутки
 4–7 суток — 1 650 ₽/сутки
 от 8 суток — 1 600 ₽/сутки
+📌 Условия аренды
 Топливо и другие расходные материалы оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Напишите в чат Авито даты аренды и суммарную мощность приборов — проверим доступность и подскажем по нагрузке.</x:v>
@@ -1502,11 +1504,13 @@
       <x:c r="F6" s="9" t="str">
         <x:v>Бензогенератор FUBAG BS 6600 A ES в аренду в Калининграде для временного электроснабжения инструмента и света на объекте.
 Цена в объявлении — 1 250 ₽/сутки при аренде от 8 суток.
+📋 Характеристики
 Номинальная мощность — 6 кВт, сеть 220 В. Есть электростартер и цифровой дисплей; бак 25 л, две розетки 16 А и одна 32 А.
-Стоимость аренды за сутки:
+💰 Стоимость аренды за сутки:
 1–2 суток — 1 800 ₽/сутки
 3–7 суток — 1 300 ₽/сутки
 от 8 суток — 1 250 ₽/сутки
+📌 Условия аренды
 Топливо и другие расходные материалы оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Напишите в чат Авито нужные даты и мощность подключаемых приборов — уточним наличие и подходящую нагрузку.</x:v>
@@ -1544,11 +1548,13 @@
       <x:c r="F7" s="9" t="str">
         <x:v>Прокат бензинового генератора FUBAG BS 3300 A ES в Калининграде для питания инструмента и освещения там, где нет сети.
 Цена в объявлении — 950 ₽/сутки при аренде от 8 суток.
+📋 Характеристики
 Номинальная мощность — 3 кВт при 220 В. Электростартер, цифровой дисплей, бак 15 л и две розетки 16 А; параметры нагрузки согласуем до выдачи.
-Стоимость аренды за сутки:
+💰 Стоимость аренды за сутки:
 1–3 суток — 1 300 ₽/сутки
 4–7 суток — 1 050 ₽/сутки
 от 8 суток — 950 ₽/сутки
+📌 Условия аренды
 Топливо и другие расходные материалы оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Укажите в сообщении Авито даты и какие приборы планируете подключать — проверим доступность генератора.</x:v>
@@ -1586,11 +1592,13 @@
       <x:c r="F8" s="9" t="str">
         <x:v>Аренда бензиновой виброплиты CHAMPION PC1151FT в Калининграде для уплотнения песка, гравия и основания под брусчатку.
 Цена в объявлении — 1 900 ₽/сутки при аренде от 8 суток.
+📋 Характеристики
 Вес 103,4 кг, центробежная сила 25 кН, плита 500 × 580 мм, глубина уплотнения до 350 мм. Коврик для плитки входит в аренду бесплатно; есть транспортировочные колёса.
-Стоимость аренды за сутки:
+💰 Стоимость аренды за сутки:
 1–2 суток — 2 200 ₽/сутки
 3–7 суток — 2 000 ₽/сутки
 от 8 суток — 1 900 ₽/сутки
+📌 Условия аренды
 Топливо и другие расходные материалы оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Напишите в чат Авито даты и тип покрытия — уточним доступность виброплиты и комплектацию.</x:v>
@@ -1626,13 +1634,15 @@
         <x:v>Аренда реверсивной виброплиты CHAMPION PC1645RH</x:v>
       </x:c>
       <x:c r="F9" s="9" t="str">
-        <x:v>Реверсивная виброплита CHAMPION PC1645RH в аренду в Калининграде для уплотнения песка, гравия и подготовки основания под брусчатку.
+        <x:v>Реверсивная виброплита CHAMPION PC1645RH в аренду в Калининграде для трамбовки песка, гравия и подготовки основания под брусчатку.
 Цена в объявлении — 2 150 ₽/сутки при аренде от 8 суток.
+📋 Характеристики
 Вес 152 кг, усилие 30,5 кН, плита 730 × 450 мм, глубина уплотнения до 500 мм. Обратный ход помогает маневрировать; коврик для плитки входит в аренду бесплатно.
-Стоимость аренды за сутки:
+💰 Стоимость аренды за сутки:
 1 сутки — 2 500 ₽/сутки
 2–7 суток — 2 200 ₽/сутки
 от 8 суток — 2 150 ₽/сутки
+📌 Условия аренды
 Топливо и другие расходные материалы оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Напишите в чат Авито сроки и материал основания — проверим наличие реверсивной плиты.</x:v>
@@ -1670,11 +1680,13 @@
       <x:c r="F10" s="9" t="str">
         <x:v>Аренда строительного пылесоса DORN PRO DPVC-40STC в Калининграде для сухой и влажной уборки после строительных работ.
 Цена в объявлении — 900 ₽/сутки при аренде от 8 суток.
+📋 Характеристики
 Мощность 1 600 Вт, бак 40 л, фильтр HEPA и автоматическая очистка фильтра. Есть розетка для инструмента до 2 000 Вт и шланг 4 м — удобно при шлифовке и штроблении.
-Стоимость аренды за сутки:
+💰 Стоимость аренды за сутки:
 1–2 суток — 1 200 ₽/сутки
 3–7 суток — 1 000 ₽/сутки
 от 8 суток — 900 ₽/сутки
+📌 Условия аренды
 Мешок для обычной уборки не включён. При штроблении и шлифовке расход мешка оплачивается отдельно; остальные расходные материалы тоже оплачиваются отдельно, если потребуются.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Напишите в чат Авито даты и тип уборки — проверим доступность пылесоса и уточним расход мешков.</x:v>
@@ -1712,11 +1724,13 @@
       <x:c r="F11" s="9" t="str">
         <x:v>Перфоратор Makita HR3011FCJ SDS-Plus в аренду в Калининграде для сверления дерева и металла, ударного сверления бетона и долбления.
 Цена в объявлении — 800 ₽/сутки при аренде от 8 суток.
+📋 Характеристики
 Мощность 1 050 Вт, удар 3,9 Дж, сверление бетона до 30 мм. AVT снижает вибрацию, подсветка помогает при слабом освещении; боковая рукоятка, ограничитель глубины и кейс в комплекте.
-Стоимость аренды за сутки:
+💰 Стоимость аренды за сутки:
 1–3 суток — 1 100 ₽/сутки
 4–7 суток — 900 ₽/сутки
 от 8 суток — 800 ₽/сутки
+📌 Условия аренды
 Буры, коронки и другие расходные материалы, если понадобятся, оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Укажите в сообщении Авито даты, материал и диаметр отверстий — проверим наличие перфоратора.</x:v>
@@ -1754,11 +1768,13 @@
       <x:c r="F12" s="9" t="str">
         <x:v>Аренда отбойного молотка Makita HM1203C в Калининграде для демонтажа бетона, кирпича и камня.
 Цена в объявлении — 1 050 ₽/сутки при аренде от 8 суток.
+📋 Характеристики
 Сетевой инструмент 1 510 Вт с ударом 19,1 Дж и патроном SDS-Max. Частоту ударов можно регулировать от 950 до 1 900 в минуту; долото ставится в 12 положениях.
-Стоимость аренды за сутки:
+💰 Стоимость аренды за сутки:
 1 сутки — 1 300 ₽/сутки
 2–7 суток — 1 100 ₽/сутки
 от 8 суток — 1 050 ₽/сутки
+📌 Условия аренды
 Расходные материалы для работ, если потребуются, оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Напишите в чат Авито даты и что нужно демонтировать — уточним доступность и комплектацию.</x:v>
@@ -1796,11 +1812,13 @@
       <x:c r="F13" s="9" t="str">
         <x:v>Воздушный компрессор FoxWeld AEROMAX 480/100 в аренду в Калининграде для работы с пневмоинструментом.
 Цена в объявлении — 1 400 ₽/сутки при аренде от 7 суток.
+📋 Характеристики
 Ресивер 100 л, производительность 480 л/мин, давление до 8 бар. Масляный ременной компрессор работает от 220 В; есть регулировка давления и защита от перегрева.
-Стоимость аренды за сутки:
+💰 Стоимость аренды за сутки:
 1–2 суток — 1 800 ₽/сутки
 3–6 суток — 1 550 ₽/сутки
 от 7 суток — 1 400 ₽/сутки
+📌 Условия аренды
 Расходные материалы для работ, если потребуются, оплачиваются отдельно; состав комплекта согласуем до выдачи.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Напишите в чат Авито даты и какой пневмоинструмент хотите подключить — проверим наличие и совместимость.</x:v>
@@ -1838,11 +1856,13 @@
       <x:c r="F14" s="9" t="str">
         <x:v>Аренда шлифмашины для стен и потолков DORN PRO DPDS-750 («жираф») в Калининграде для гипсокартона и оштукатуренных поверхностей.
 Цена в объявлении — 950 ₽/сутки при аренде от 8 суток.
+📋 Характеристики
 Диск 225 мм, мощность 750 Вт, регулировка 600–1 850 об/мин. Есть подсветка зоны работы и подключение к пылесосу для отвода пыли.
-Стоимость аренды за сутки:
+💰 Стоимость аренды за сутки:
 1–2 суток — 1 100 ₽/сутки
 3–7 суток — 1 000 ₽/сутки
 от 8 суток — 950 ₽/сутки
+📌 Условия аренды
 Шлифлисты (абразивы) и другие расходные материалы оплачиваются отдельно. Необходимость пылесоса уточним при оформлении.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Укажите в сообщении Авито даты и площадь шлифовки — проверим доступность машины и подходящие абразивы.</x:v>
@@ -1880,11 +1900,13 @@
       <x:c r="F15" s="9" t="str">
         <x:v>Аренда погружного фекального насоса Oasis F-1500/13R с измельчителем в Калининграде для откачки грязной воды и канализационных стоков.
 Цена в объявлении — 750 ₽/сутки при аренде от 8 суток.
+📋 Характеристики
 Мощность 1 500 Вт, производительность до 24 900 л/ч, напор до 13 м. В комплекте два рукава по 20 м диаметром 2″, хомуты, соединители и трос.
-Стоимость аренды за сутки:
+💰 Стоимость аренды за сутки:
 1–3 суток — 950 ₽/сутки
 4–7 суток — 800 ₽/сутки
 от 8 суток — 750 ₽/сутки
+📌 Условия аренды
 Для канализационных и фекальных стоков санитарная очистка стоит дополнительно 1 000 ₽. Если очистите насос перед возвратом самостоятельно, этой доплаты нет. Расходные материалы для работ, если понадобятся, оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Напишите в чат Авито, что нужно откачать, глубину и даты — уточним доступность насоса и условия очистки.</x:v>
@@ -1922,11 +1944,13 @@
       <x:c r="F16" s="9" t="str">
         <x:v>Бетономешалка ПРОФМАШ Б180 в аренду в Калининграде для приготовления бетона, кладочного или штукатурного раствора.
 Цена в объявлении — 750 ₽/сутки при аренде от 7 суток.
+📋 Характеристики
 Объём бака 160 л, готовой смеси — до 90 л; мощность 700 Вт, питание 220 В. Чугунный венец и транспортировочные колёса.
-Стоимость аренды за сутки:
+💰 Стоимость аренды за сутки:
 1–2 суток — 1 050 ₽/сутки
 3–6 суток — 850 ₽/сутки
 от 7 суток — 750 ₽/сутки
+📌 Условия аренды
 Верните бетоносмеситель очищенным. Очистка при возврате с застывшим раствором стоит 1 500 ₽; расходные материалы для работ оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Напишите в чат Авито даты и объём работ — проверим доступность бетономешалки.</x:v>
@@ -1964,11 +1988,13 @@
       <x:c r="F17" s="9" t="str">
         <x:v>Аренда промышленного осушителя воздуха BALLU BDI-50L в Калининграде для сушки помещений после ремонта и строительных работ.
 Цена в объявлении — 550 ₽/сутки при аренде от 8 суток.
+📋 Характеристики
 Осушение до 50 л/сутки зависит от температуры и влажности. Воздухообмен 350 м³/ч, бак 7 л; встроенные гигрометр и гигростат помогают контролировать влажность.
-Стоимость аренды за сутки:
+💰 Стоимость аренды за сутки:
 1–3 суток — 650 ₽/сутки
 4–7 суток — 600 ₽/сутки
 от 8 суток — 550 ₽/сутки
+📌 Условия аренды
 Расходные материалы для ваших работ, если потребуются, оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Укажите в сообщении Авито площадь помещения, условия влажности и даты — проверим доступность осушителя.</x:v>
@@ -2006,11 +2032,13 @@
       <x:c r="F18" s="9" t="str">
         <x:v>Аренда алюминиевой стремянки DORN PRO 115594 на 4 ступени в Калининграде для ремонта, монтажа и работ внутри помещения.
 Цена в объявлении — 240 ₽/сутки при аренде от 8 суток.
+📋 Характеристики
 Высота площадки 0,91 м, допустимая нагрузка до 150 кг. Ребристые ступени, поручень и противоскользящие опоры; в сложенном виде толщина всего 55 мм.
-Стоимость аренды за сутки:
+💰 Стоимость аренды за сутки:
 1–3 суток — 330 ₽/сутки
 4–7 суток — 270 ₽/сутки
 от 8 суток — 240 ₽/сутки
+📌 Условия аренды
 Расходные материалы для ваших работ, если потребуются, оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Напишите в чат Авито нужную высоту и даты — проверим доступность стремянки.</x:v>
@@ -2048,11 +2076,13 @@
       <x:c r="F19" s="9" t="str">
         <x:v>Прокат алюминиевой стремянки Новая Высота 200 на 10 ступеней в Калининграде для ремонта и монтажных работ на высоте.
 Цена в объявлении — 500 ₽/сутки при аренде от 8 суток.
+📋 Характеристики
 Площадка на высоте 2,17 м, допустимая нагрузка до 180 кг. Есть органайзер для инструмента, крюк для ведра, рифлёные ступени и противоскользящие опоры.
-Стоимость аренды за сутки:
+💰 Стоимость аренды за сутки:
 1–3 суток — 650 ₽/сутки
 4–7 суток — 550 ₽/сутки
 от 8 суток — 500 ₽/сутки
+📌 Условия аренды
 Расходные материалы для ваших работ, если потребуются, оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Укажите в сообщении Авито нужную высоту и даты — проверим доступность стремянки.</x:v>
@@ -2090,11 +2120,13 @@
       <x:c r="F20" s="9" t="str">
         <x:v>Аккумуляторная дрель-шуруповёрт Makita DDF484RME в аренду в Калининграде для крепежа и сверления дерева, металла и пластика.
 Цена в объявлении — 600 ₽/сутки при аренде от 8 суток.
+📋 Характеристики
 Бесщёточный двигатель 18 В, момент 54 Н·м, две скорости и подсветка. В комплекте два аккумулятора 4,0 А·ч, зарядное устройство и кейс; ударного режима нет.
-Стоимость аренды за сутки:
+💰 Стоимость аренды за сутки:
 1–3 суток — 700 ₽/сутки
 4–7 суток — 650 ₽/сутки
 от 8 суток — 600 ₽/сутки
+📌 Условия аренды
 Свёрла и другие расходные материалы оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Напишите в чат Авито даты и материал для сверления — уточним доступность шуруповёрта.</x:v>
@@ -2132,11 +2164,13 @@
       <x:c r="F21" s="9" t="str">
         <x:v>Аренда строительного фена Makita HG5030K в Калининграде для сушки и размягчения материалов при ремонте.
 Цена в объявлении — 450 ₽/сутки при аренде от 8 суток.
+📋 Характеристики
 Технический фен 1 600 Вт с режимами 350 и 500 °C, потоком воздуха 300 и 500 л/мин. В комплекте четыре насадки и кейс; возможна стационарная установка.
-Стоимость аренды за сутки:
+💰 Стоимость аренды за сутки:
 1–2 суток — 550 ₽/сутки
 3–7 суток — 500 ₽/сутки
 от 8 суток — 450 ₽/сутки
+📌 Условия аренды
 Расходные материалы для ваших работ, если потребуются, оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Укажите в сообщении Авито материал, задачу и даты — проверим доступность термофена.</x:v>
@@ -2157,7 +2191,7 @@
         <x:v>450</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="285" customHeight="1">
+    <x:row r="22" ht="330" customHeight="1">
       <x:c r="A22" s="8" t="str">
         <x:v>Предложение услуг</x:v>
       </x:c>
@@ -2174,11 +2208,13 @@
       <x:c r="F22" s="9" t="str">
         <x:v>Бензорез CHAMPION CP350 в аренду в Калининграде для резки бетона, асфальта и камня; металл режется с подходящим диском.
 Цена в объявлении — 2 000 ₽/сутки при аренде от 8 суток.
+📋 Характеристики
 Мощность 3,5 кВт, диск 350 мм, глубина реза до 125 мм. Возможна сухая и мокрая резка с подходящим диском; предусмотрена подача воды.
-Стоимость аренды за сутки:
+💰 Стоимость аренды за сутки:
 1–2 суток — 2 250 ₽/сутки
 3–7 суток — 2 100 ₽/сутки
 от 8 суток — 2 000 ₽/сутки
+📌 Условия аренды
 Топливо и прочие расходные материалы оплачиваются отдельно. Износ нашего алмазного диска 350 мм оплачивается по факту — 1 000 ₽/мм; минимальное списание 0,5 мм = 500 ₽. При использовании своего совместимого диска доплаты за износ нет.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Напишите в чат Авито материал, глубину реза и даты. Если у вас свой диск, укажите его параметры — уточним совместимость и доступность бензореза.</x:v>
@@ -2216,11 +2252,13 @@
       <x:c r="F23" s="9" t="str">
         <x:v>Аренда штробореза ЗУБР ЗШ-П65-2700 ПСТК в Калининграде для прокладки каналов в бетоне и кирпиче.
 Цена в объявлении — 1 000 ₽/сутки при аренде от 8 суток.
+📋 Характеристики
 Бороздодел 2 700 Вт работает с двумя дисками 230 мм: глубина реза до 65 мм, ширина штробы 4,3–40 мм. Есть плавный пуск и подключение к пылесосу.
-Стоимость аренды за сутки:
+💰 Стоимость аренды за сутки:
 1–3 суток — 1 400 ₽/сутки
 4–7 суток — 1 100 ₽/сутки
 от 8 суток — 1 000 ₽/сутки
+📌 Условия аренды
 Подбор дисков и условия оплаты их износа согласуем до выдачи. Строительный пылесос арендуется отдельно; расходные материалы оплачиваются отдельно.
 Без залога. Самовывоз и самостоятельный возврат бесплатны, адрес и время согласуем. Доставка по Калининграду — 900 ₽, обратный вывоз — ещё 900 ₽. По области условия согласуем отдельно.
 Напишите в чат Авито материал стены, размеры штробы и даты — проверим доступность инструмента.</x:v>
@@ -2257,10 +2295,10 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="R507035b5d2dd43ae"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="Rcfc385d250aa44f1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="R28a0f27ed7ec49e2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="Rac306d85ae4c477c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="Rf03196e51a83442f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="Rba82cb8a6f73475c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="Rdc7bb24ddc6c4cda"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="Rb8e57ae6b174471c"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Clarify equipment weights in Avito XLSX feed
</commit_message>
<xml_diff>
--- a/stroyrent39-avito-19-2026-09-30.xlsx
+++ b/stroyrent39-avito-19-2026-09-30.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" r:id="Re3953f24f6a84d98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объявления" sheetId="2" r:id="Ra4bd3f90f98046ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Справочники" sheetId="3" r:id="R1a8b3dc00730408a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" r:id="Rd863664f913e4f3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объявления" sheetId="2" r:id="R25434d133bbd46d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Справочники" sheetId="3" r:id="Rf1debd096a974eeb"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="Instructions" localSheetId="0">Инструкция!$1:$50</x:definedName>
@@ -1303,13 +1303,13 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="R128ae135a3fd4456"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="R9004f87e3b364176"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="R2860d14a3a4f486e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="R3b118e96bd5e429e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="Rc2363564df274ea8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="R9a99d80364b04a27"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="R2eb6697129c946a1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="Rd0f5f6a6c61a4b30"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="R53e580cff72b4812"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="R23c71422d1e54af8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="R297da29b93864aee"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="Rcc231c7ad9484043"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="R3a14c93792fb41d2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="R506fd808430a4403"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1590,10 +1590,10 @@
         <x:v>Аренда виброплиты CHAMPION PC1151FT для трамбовки</x:v>
       </x:c>
       <x:c r="F8" s="9" t="str">
-        <x:v>Аренда бензиновой виброплиты CHAMPION PC1151FT в Калининграде для уплотнения песка, гравия и основания под брусчатку.
+        <x:v>Аренда бензиновой виброплиты CHAMPION PC1151FT в Калининграде для уплотнения песка, гравия и основания под брусчатку. Вес плиты — 103,4 кг.
 Цена в объявлении — 1 900 ₽/сутки при аренде от 8 суток.
 📋 Характеристики
-Вес 103,4 кг, центробежная сила 25 кН, плита 500 × 580 мм, глубина уплотнения до 350 мм. Коврик для плитки входит в аренду бесплатно; есть транспортировочные колёса.
+Центробежная сила 25 кН, плита 500 × 580 мм, глубина уплотнения до 350 мм. Коврик для плитки входит в аренду бесплатно; есть транспортировочные колёса.
 💰 Стоимость аренды за сутки:
 1–2 суток — 2 200 ₽/сутки
 3–7 суток — 2 000 ₽/сутки
@@ -1634,10 +1634,10 @@
         <x:v>Аренда реверсивной виброплиты CHAMPION PC1645RH</x:v>
       </x:c>
       <x:c r="F9" s="9" t="str">
-        <x:v>Реверсивная виброплита CHAMPION PC1645RH в аренду в Калининграде для трамбовки песка, гравия и подготовки основания под брусчатку.
+        <x:v>Реверсивная виброплита CHAMPION PC1645RH в аренду в Калининграде для трамбовки песка, гравия и подготовки основания под брусчатку. Вес плиты — 152 кг.
 Цена в объявлении — 2 150 ₽/сутки при аренде от 8 суток.
 📋 Характеристики
-Вес 152 кг, усилие 30,5 кН, плита 730 × 450 мм, глубина уплотнения до 500 мм. Обратный ход помогает маневрировать; коврик для плитки входит в аренду бесплатно.
+Усилие 30,5 кН, плита 730 × 450 мм, глубина уплотнения до 500 мм. Обратный ход помогает маневрировать; коврик для плитки входит в аренду бесплатно.
 💰 Стоимость аренды за сутки:
 1 сутки — 2 500 ₽/сутки
 2–7 суток — 2 200 ₽/сутки
@@ -2295,10 +2295,10 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="Rf03196e51a83442f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="Rba82cb8a6f73475c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="Rdc7bb24ddc6c4cda"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="Rb8e57ae6b174471c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="R89df76d8a09543e6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="R86e05f22939c419a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="R04d78495e3b14fff"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="Rc541bd93ee02490b"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>